<commit_message>
Update curated NID-MS training workbook
Doubles the NID-MS example count (5 -> 10) after re-import. Header
row was already on row 1, so no parser change needed this time.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Training Data/Automation/NID-MS.xlsx
+++ b/Training Data/Automation/NID-MS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\GitHub\SMS_Automation\Training Data\Automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Documents\GitHub\SMS_Automation\Training Data\Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DDFF21E-29DB-4440-B2DD-FBA645BF5D15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D23F4BAB-EF59-44BF-974B-304F9D7B2D6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1080" windowWidth="14400" windowHeight="8230" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="NID-MS" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="17">
   <si>
     <t>SL No</t>
   </si>
@@ -48,30 +48,44 @@
     <t>NID-MS 19907917652000048</t>
   </si>
   <si>
-    <t xml:space="preserve">NID: 19907917652000048 8801744888421 [GP]
-NID 19907917652000048 No data found - Banglalink
-</t>
-  </si>
-  <si>
     <t>NID-MS 3758355105</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NID: 3758355105
-MSISDN: 
-8801610420628
-8801610027553 [Robi]
-</t>
   </si>
   <si>
     <t>NID: 19907917652000048
 8801744888421 [GP]</t>
+  </si>
+  <si>
+    <t>NID 19907917652000048 No data found - Banglalink</t>
+  </si>
+  <si>
+    <t>NID-MS 19787918785632712</t>
+  </si>
+  <si>
+    <t>NID: 19787918785632712
+MSISDN: 
+8801872664308 [Robi]</t>
+  </si>
+  <si>
+    <t>NID-MS 19700619452170146</t>
+  </si>
+  <si>
+    <t>NID 19700619452170146 MSISDN: 8801904897498 - Banglalink</t>
+  </si>
+  <si>
+    <t>NID: 3758355105
+MSISDN: 8801610420628
+8801610027553 [Robi]</t>
+  </si>
+  <si>
+    <t>NID: 19907917652000048 8801744888421 [GP]
+NID 19907917652000048 No data found - Banglalink</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -634,8 +648,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B2D1F3A7-AB7D-4F67-A1A7-000BAD65A856}" name="Table1" displayName="Table1" ref="A1:C6" totalsRowShown="0">
-  <autoFilter ref="A1:C6" xr:uid="{B2D1F3A7-AB7D-4F67-A1A7-000BAD65A856}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B2D1F3A7-AB7D-4F67-A1A7-000BAD65A856}" name="Table1" displayName="Table1" ref="A1:C11" totalsRowShown="0">
+  <autoFilter ref="A1:C11" xr:uid="{B2D1F3A7-AB7D-4F67-A1A7-000BAD65A856}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{2D60EBF0-36FB-4E1F-94B1-14A65144EC0B}" name="SL No" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{7674A791-190E-4066-BFE1-7624D6ED49A2}" name="Request" dataDxfId="1"/>
@@ -962,15 +976,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="8.81640625" style="1"/>
-    <col min="2" max="2" width="24.31640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.875" style="1"/>
+    <col min="2" max="2" width="24.375" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="59" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -981,7 +995,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="44.25" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:3" ht="42.75">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -992,7 +1006,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1003,7 +1017,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="44.25" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:3" ht="28.5">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1011,21 +1025,21 @@
         <v>7</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="73.75" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:3" ht="42.75">
       <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:3" ht="28.5">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1033,7 +1047,62 @@
         <v>7</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="28.5">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="42.75">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>11</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>